<commit_message>
data: updated ratings - below budget label
</commit_message>
<xml_diff>
--- a/Fleet_Routes_Analytics.xlsx
+++ b/Fleet_Routes_Analytics.xlsx
@@ -548,7 +548,7 @@
         <v>0.094</v>
       </c>
       <c r="N2" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="3">
@@ -580,7 +580,7 @@
         <v>0.146</v>
       </c>
       <c r="N3" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="4">
@@ -624,7 +624,7 @@
         <v>79</v>
       </c>
       <c r="N4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -656,7 +656,7 @@
         <v>0.802</v>
       </c>
       <c r="N5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -688,7 +688,7 @@
         <v>1.123</v>
       </c>
       <c r="N6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -720,7 +720,7 @@
         <v>1.835</v>
       </c>
       <c r="N7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="8">
@@ -752,7 +752,7 @@
         <v>2.064</v>
       </c>
       <c r="N8" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="9">
@@ -784,7 +784,7 @@
         <v>2.639</v>
       </c>
       <c r="N9" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="10">
@@ -816,7 +816,7 @@
         <v>3.049</v>
       </c>
       <c r="N10" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="11">
@@ -848,7 +848,7 @@
         <v>3.233</v>
       </c>
       <c r="N11" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="12">
@@ -880,7 +880,7 @@
         <v>3.419</v>
       </c>
       <c r="N12" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="13">
@@ -912,7 +912,7 @@
         <v>3.809</v>
       </c>
       <c r="N13" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="14">
@@ -944,7 +944,7 @@
         <v>3.837</v>
       </c>
       <c r="N14" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="15">
@@ -976,7 +976,7 @@
         <v>3.948</v>
       </c>
       <c r="N15" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="16">
@@ -1008,7 +1008,7 @@
         <v>4.17</v>
       </c>
       <c r="N16" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="17">
@@ -1040,7 +1040,7 @@
         <v>4.734</v>
       </c>
       <c r="N17" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="18">
@@ -1072,7 +1072,7 @@
         <v>4.765</v>
       </c>
       <c r="N18" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="19">
@@ -1104,7 +1104,7 @@
         <v>5.077</v>
       </c>
       <c r="N19" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="20">
@@ -1136,7 +1136,7 @@
         <v>5.64</v>
       </c>
       <c r="N20" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="21">
@@ -1168,7 +1168,7 @@
         <v>5.986</v>
       </c>
       <c r="N21" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="22">
@@ -1200,7 +1200,7 @@
         <v>6.77</v>
       </c>
       <c r="N22" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="23">
@@ -1232,7 +1232,7 @@
         <v>7.482</v>
       </c>
       <c r="N23" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="24">
@@ -1264,7 +1264,7 @@
         <v>8.004</v>
       </c>
       <c r="N24" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="25">
@@ -1296,7 +1296,7 @@
         <v>10.272</v>
       </c>
       <c r="N25" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="26">
@@ -1328,7 +1328,7 @@
         <v>14.437</v>
       </c>
       <c r="N26" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="27">
@@ -1360,7 +1360,7 @@
         <v>25.282</v>
       </c>
       <c r="N27" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="28">
@@ -1392,7 +1392,7 @@
         <v>41.898</v>
       </c>
       <c r="N28" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="29">
@@ -1436,7 +1436,7 @@
         <v>17350</v>
       </c>
       <c r="N29" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -1579,7 +1579,7 @@
         <v>3.886</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -1626,7 +1626,7 @@
         <v>2.974</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -1673,7 +1673,7 @@
         <v>11.099</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -1816,7 +1816,7 @@
         <v>0.126</v>
       </c>
       <c r="T2" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="3">
@@ -1872,7 +1872,7 @@
         <v>5.701</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -1919,7 +1919,7 @@
         <v>3.998</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -1969,7 +1969,7 @@
         <v>2.711</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -2019,7 +2019,7 @@
         <v>3.627</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -2162,7 +2162,7 @@
         <v>4.879</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -2212,7 +2212,7 @@
         <v>6.14</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -2268,7 +2268,7 @@
         <v>3.142</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -2324,7 +2324,7 @@
         <v>4.129</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -2380,7 +2380,7 @@
         <v>6.735</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -2436,7 +2436,7 @@
         <v>4.359</v>
       </c>
       <c r="T7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="8">
@@ -2498,7 +2498,7 @@
         <v>3.759</v>
       </c>
       <c r="T8" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="9">
@@ -2560,7 +2560,7 @@
         <v>2056.881</v>
       </c>
       <c r="T9" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -2706,7 +2706,7 @@
         <v>0.058</v>
       </c>
       <c r="T2" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="3">
@@ -2762,7 +2762,7 @@
         <v>8.307</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -2809,7 +2809,7 @@
         <v>11.408</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -2865,7 +2865,7 @@
         <v>6.988</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -2912,7 +2912,7 @@
         <v>69.611</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -2959,7 +2959,7 @@
         <v>69.333</v>
       </c>
       <c r="T7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -3102,7 +3102,7 @@
         <v>6.952</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -3158,7 +3158,7 @@
         <v>4.49</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -3214,7 +3214,7 @@
         <v>8.373</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -3261,7 +3261,7 @@
         <v>1.957</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -3308,7 +3308,7 @@
         <v>3.988</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -3358,7 +3358,7 @@
         <v>3.988</v>
       </c>
       <c r="T7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -3501,7 +3501,7 @@
         <v>2.335</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -3557,7 +3557,7 @@
         <v>4.317</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -3604,7 +3604,7 @@
         <v>3.709</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -3756,7 +3756,7 @@
         <v>1.165</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -3803,7 +3803,7 @@
         <v>3.006</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -3859,7 +3859,7 @@
         <v>1.748</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -3915,7 +3915,7 @@
         <v>10.169</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -3971,7 +3971,7 @@
         <v>9.666</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -4117,7 +4117,7 @@
         <v>14.437</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -4167,7 +4167,7 @@
         <v>14.437</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -4310,7 +4310,7 @@
         <v>1.952</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -4357,7 +4357,7 @@
         <v>4.998</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -4413,7 +4413,7 @@
         <v>4.561</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -4559,7 +4559,7 @@
         <v>0.659</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -4609,7 +4609,7 @@
         <v>2.512</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -4665,7 +4665,7 @@
         <v>5.916</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -4783,7 +4783,7 @@
         <v>0.146</v>
       </c>
       <c r="P2" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="3">
@@ -4821,7 +4821,7 @@
         <v>0.802</v>
       </c>
       <c r="P3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -4859,7 +4859,7 @@
         <v>1.123</v>
       </c>
       <c r="P4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -4897,7 +4897,7 @@
         <v>1.835</v>
       </c>
       <c r="P5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -4935,7 +4935,7 @@
         <v>3.233</v>
       </c>
       <c r="P6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -4973,7 +4973,7 @@
         <v>3.709</v>
       </c>
       <c r="P7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="8">
@@ -5011,7 +5011,7 @@
         <v>3.734</v>
       </c>
       <c r="P8" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="9">
@@ -5049,7 +5049,7 @@
         <v>3.837</v>
       </c>
       <c r="P9" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="10">
@@ -5087,7 +5087,7 @@
         <v>3.915</v>
       </c>
       <c r="P10" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="11">
@@ -5125,7 +5125,7 @@
         <v>4.325</v>
       </c>
       <c r="P11" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="12">
@@ -5175,7 +5175,7 @@
         <v>447.7</v>
       </c>
       <c r="P12" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="13">
@@ -5213,7 +5213,7 @@
         <v>4.576</v>
       </c>
       <c r="P13" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="14">
@@ -5251,7 +5251,7 @@
         <v>4.867</v>
       </c>
       <c r="P14" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="15">
@@ -5289,7 +5289,7 @@
         <v>5.029</v>
       </c>
       <c r="P15" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="16">
@@ -5327,7 +5327,7 @@
         <v>5.916</v>
       </c>
       <c r="P16" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="17">
@@ -5365,7 +5365,7 @@
         <v>5.986</v>
       </c>
       <c r="P17" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="18">
@@ -5403,7 +5403,7 @@
         <v>6.815</v>
       </c>
       <c r="P18" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="19">
@@ -5441,7 +5441,7 @@
         <v>6.987</v>
       </c>
       <c r="P19" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="20">
@@ -5479,7 +5479,7 @@
         <v>7.482</v>
       </c>
       <c r="P20" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="21">
@@ -5517,7 +5517,7 @@
         <v>8.004</v>
       </c>
       <c r="P21" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="22">
@@ -5555,7 +5555,7 @@
         <v>10.169</v>
       </c>
       <c r="P22" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="23">
@@ -5593,7 +5593,7 @@
         <v>14.39</v>
       </c>
       <c r="P23" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="24">
@@ -5631,7 +5631,7 @@
         <v>14.437</v>
       </c>
       <c r="P24" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="25">
@@ -5669,7 +5669,7 @@
         <v>33.13</v>
       </c>
       <c r="P25" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="26">
@@ -5707,7 +5707,7 @@
         <v>62.563</v>
       </c>
       <c r="P26" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="27">
@@ -5757,7 +5757,7 @@
         <v>205688.1</v>
       </c>
       <c r="P27" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="28">
@@ -5795,7 +5795,7 @@
         <v>0.058</v>
       </c>
       <c r="P28" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="29">
@@ -5833,7 +5833,7 @@
         <v>0.094</v>
       </c>
       <c r="P29" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="30">
@@ -5883,7 +5883,7 @@
         <v>125.3</v>
       </c>
       <c r="P30" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="31">
@@ -5921,7 +5921,7 @@
         <v>1.586</v>
       </c>
       <c r="P31" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="32">
@@ -5959,7 +5959,7 @@
         <v>1.977</v>
       </c>
       <c r="P32" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="33">
@@ -5997,7 +5997,7 @@
         <v>2.044</v>
       </c>
       <c r="P33" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="34">
@@ -6035,7 +6035,7 @@
         <v>2.064</v>
       </c>
       <c r="P34" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="35">
@@ -6073,7 +6073,7 @@
         <v>2.609</v>
       </c>
       <c r="P35" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="36">
@@ -6111,7 +6111,7 @@
         <v>3.129</v>
       </c>
       <c r="P36" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="37">
@@ -6149,7 +6149,7 @@
         <v>3.326</v>
       </c>
       <c r="P37" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="38">
@@ -6187,7 +6187,7 @@
         <v>3.871</v>
       </c>
       <c r="P38" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="39">
@@ -6225,7 +6225,7 @@
         <v>4.066</v>
       </c>
       <c r="P39" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="40">
@@ -6263,7 +6263,7 @@
         <v>4.325</v>
       </c>
       <c r="P40" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="41">
@@ -6301,7 +6301,7 @@
         <v>4.341</v>
       </c>
       <c r="P41" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="42">
@@ -6339,7 +6339,7 @@
         <v>4.807</v>
       </c>
       <c r="P42" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="43">
@@ -6377,7 +6377,7 @@
         <v>6.623</v>
       </c>
       <c r="P43" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="44">
@@ -6415,7 +6415,7 @@
         <v>6.952</v>
       </c>
       <c r="P44" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="45">
@@ -6453,7 +6453,7 @@
         <v>1.165</v>
       </c>
       <c r="P45" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="46">
@@ -6491,7 +6491,7 @@
         <v>2.681</v>
       </c>
       <c r="P46" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="47">
@@ -6529,7 +6529,7 @@
         <v>2.705</v>
       </c>
       <c r="P47" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="48">
@@ -6567,7 +6567,7 @@
         <v>2.881</v>
       </c>
       <c r="P48" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="49">
@@ -6605,7 +6605,7 @@
         <v>4.49</v>
       </c>
       <c r="P49" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="50">
@@ -6643,7 +6643,7 @@
         <v>5.471</v>
       </c>
       <c r="P50" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="51">
@@ -6681,7 +6681,7 @@
         <v>5.6</v>
       </c>
       <c r="P51" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -6833,7 +6833,7 @@
         <v>3.457</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -6889,7 +6889,7 @@
         <v>5.225</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -6945,7 +6945,7 @@
         <v>4.7</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -6992,7 +6992,7 @@
         <v>15.823</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -7048,7 +7048,7 @@
         <v>0.437</v>
       </c>
       <c r="T6" t="str">
-        <v>⚠️ Slightly High</v>
+        <v>✅ Within Allocation</v>
       </c>
     </row>
   </sheetData>
@@ -7191,7 +7191,7 @@
         <v>1.504</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -7238,7 +7238,7 @@
         <v>2.639</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -7288,7 +7288,7 @@
         <v>1.363</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -7434,7 +7434,7 @@
         <v>1.1</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -7490,7 +7490,7 @@
         <v>3.028</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -7642,7 +7642,7 @@
         <v>2.681</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -7698,7 +7698,7 @@
         <v>1.977</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -7754,7 +7754,7 @@
         <v>5.828</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -7810,7 +7810,7 @@
         <v>6.857</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -7857,7 +7857,7 @@
         <v>22.956</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -7904,7 +7904,7 @@
         <v>23.583</v>
       </c>
       <c r="T7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="8">
@@ -7951,7 +7951,7 @@
         <v>23.583</v>
       </c>
       <c r="T8" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="9">
@@ -7998,7 +7998,7 @@
         <v>3.535</v>
       </c>
       <c r="T9" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -8150,7 +8150,7 @@
         <v>0.094</v>
       </c>
       <c r="T2" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
   </sheetData>
@@ -8292,7 +8292,7 @@
         <v>9.211</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -8339,7 +8339,7 @@
         <v>3.098</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -8395,7 +8395,7 @@
         <v>4.644</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -8451,7 +8451,7 @@
         <v>2.152</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -8498,7 +8498,7 @@
         <v>1.618</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -8545,7 +8545,7 @@
         <v>2.219</v>
       </c>
       <c r="T7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="8">
@@ -8592,7 +8592,7 @@
         <v>2.278</v>
       </c>
       <c r="T8" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="9">
@@ -8642,7 +8642,7 @@
         <v>8.469</v>
       </c>
       <c r="T9" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -8794,7 +8794,7 @@
         <v>0.146</v>
       </c>
       <c r="T2" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
   </sheetData>
@@ -8945,7 +8945,7 @@
         <v>6.623</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -9001,7 +9001,7 @@
         <v>7.629</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -9057,7 +9057,7 @@
         <v>7.884</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -9113,7 +9113,7 @@
         <v>8.986</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -9169,7 +9169,7 @@
         <v>4.788</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -9225,7 +9225,7 @@
         <v>4.788</v>
       </c>
       <c r="T7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -9368,7 +9368,7 @@
         <v>3.129</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -9415,7 +9415,7 @@
         <v>4.867</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -9558,7 +9558,7 @@
         <v>5.6</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -9605,7 +9605,7 @@
         <v>3.381</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -9652,7 +9652,7 @@
         <v>3.381</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -9699,7 +9699,7 @@
         <v>5.436</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -9746,7 +9746,7 @@
         <v>6.453</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -9793,7 +9793,7 @@
         <v>7.214</v>
       </c>
       <c r="T7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="8">
@@ -9840,7 +9840,7 @@
         <v>4.377</v>
       </c>
       <c r="T8" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="9">
@@ -9887,7 +9887,7 @@
         <v>4.377</v>
       </c>
       <c r="T9" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="10">
@@ -9934,7 +9934,7 @@
         <v>5.777</v>
       </c>
       <c r="T10" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="11">
@@ -9990,7 +9990,7 @@
         <v>1.978</v>
       </c>
       <c r="T11" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -10136,7 +10136,7 @@
         <v>0.058</v>
       </c>
       <c r="T2" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="3">
@@ -10186,7 +10186,7 @@
         <v>4.195</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -10233,7 +10233,7 @@
         <v>9.211</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -10280,7 +10280,7 @@
         <v>3.886</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -10327,7 +10327,7 @@
         <v>4.879</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -10383,7 +10383,7 @@
         <v>0.043</v>
       </c>
       <c r="T7" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="8">
@@ -10430,7 +10430,7 @@
         <v>5.6</v>
       </c>
       <c r="T8" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="9">
@@ -10477,7 +10477,7 @@
         <v>2.881</v>
       </c>
       <c r="T9" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="10">
@@ -10524,7 +10524,7 @@
         <v>6.952</v>
       </c>
       <c r="T10" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="11">
@@ -10571,7 +10571,7 @@
         <v>3.381</v>
       </c>
       <c r="T11" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="12">
@@ -10618,7 +10618,7 @@
         <v>3.547</v>
       </c>
       <c r="T12" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="13">
@@ -10674,7 +10674,7 @@
         <v>1.165</v>
       </c>
       <c r="T13" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="14">
@@ -10724,7 +10724,7 @@
         <v>6.14</v>
       </c>
       <c r="T14" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="15">
@@ -10780,7 +10780,7 @@
         <v>4.036</v>
       </c>
       <c r="T15" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="16">
@@ -10827,7 +10827,7 @@
         <v>3.006</v>
       </c>
       <c r="T16" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="17">
@@ -10874,7 +10874,7 @@
         <v>2.335</v>
       </c>
       <c r="T17" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="18">
@@ -10924,7 +10924,7 @@
         <v>0.659</v>
       </c>
       <c r="T18" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="19">
@@ -10974,7 +10974,7 @@
         <v>2.609</v>
       </c>
       <c r="T19" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="20">
@@ -11030,7 +11030,7 @@
         <v>3.142</v>
       </c>
       <c r="T20" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="21">
@@ -11086,7 +11086,7 @@
         <v>6.623</v>
       </c>
       <c r="T21" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="22">
@@ -11133,7 +11133,7 @@
         <v>3.381</v>
       </c>
       <c r="T22" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="23">
@@ -11180,7 +11180,7 @@
         <v>5.231</v>
       </c>
       <c r="T23" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="24">
@@ -11236,7 +11236,7 @@
         <v>4.49</v>
       </c>
       <c r="T24" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="25">
@@ -11292,7 +11292,7 @@
         <v>2.681</v>
       </c>
       <c r="T25" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="26">
@@ -11348,7 +11348,7 @@
         <v>4.036</v>
       </c>
       <c r="T26" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="27">
@@ -11404,7 +11404,7 @@
         <v>0.534</v>
       </c>
       <c r="T27" t="str">
-        <v>⚠️ Slightly High</v>
+        <v>⚠️ Slightly Over Budget</v>
       </c>
     </row>
     <row r="28">
@@ -11451,7 +11451,7 @@
         <v>2.618</v>
       </c>
       <c r="T28" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="29">
@@ -11507,7 +11507,7 @@
         <v>1.977</v>
       </c>
       <c r="T29" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="30">
@@ -11563,7 +11563,7 @@
         <v>1.748</v>
       </c>
       <c r="T30" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="31">
@@ -11619,7 +11619,7 @@
         <v>4.317</v>
       </c>
       <c r="T31" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="32">
@@ -11669,7 +11669,7 @@
         <v>2.512</v>
       </c>
       <c r="T32" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="33">
@@ -11719,7 +11719,7 @@
         <v>2.609</v>
       </c>
       <c r="T33" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="34">
@@ -11766,7 +11766,7 @@
         <v>5.436</v>
       </c>
       <c r="T34" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="35">
@@ -11813,7 +11813,7 @@
         <v>3.129</v>
       </c>
       <c r="T35" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="36">
@@ -11869,7 +11869,7 @@
         <v>4.129</v>
       </c>
       <c r="T36" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="37">
@@ -11925,7 +11925,7 @@
         <v>8.373</v>
       </c>
       <c r="T37" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="38">
@@ -11981,7 +11981,7 @@
         <v>8.307</v>
       </c>
       <c r="T38" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="39">
@@ -12037,7 +12037,7 @@
         <v>5.828</v>
       </c>
       <c r="T39" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="40">
@@ -12093,7 +12093,7 @@
         <v>10.169</v>
       </c>
       <c r="T40" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="41">
@@ -12149,7 +12149,7 @@
         <v>5.916</v>
       </c>
       <c r="T41" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="42">
@@ -12205,7 +12205,7 @@
         <v>3.367</v>
       </c>
       <c r="T42" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="43">
@@ -12252,7 +12252,7 @@
         <v>2.974</v>
       </c>
       <c r="T43" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="44">
@@ -12308,7 +12308,7 @@
         <v>7.629</v>
       </c>
       <c r="T44" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="45">
@@ -12355,7 +12355,7 @@
         <v>6.453</v>
       </c>
       <c r="T45" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="46">
@@ -12402,7 +12402,7 @@
         <v>4.484</v>
       </c>
       <c r="T46" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="47">
@@ -12449,7 +12449,7 @@
         <v>4.867</v>
       </c>
       <c r="T47" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="48">
@@ -12505,7 +12505,7 @@
         <v>6.735</v>
       </c>
       <c r="T48" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="49">
@@ -12561,7 +12561,7 @@
         <v>7.884</v>
       </c>
       <c r="T49" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="50">
@@ -12608,7 +12608,7 @@
         <v>4.641</v>
       </c>
       <c r="T50" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="51">
@@ -12664,7 +12664,7 @@
         <v>0.094</v>
       </c>
       <c r="T51" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="52">
@@ -12720,7 +12720,7 @@
         <v>6.857</v>
       </c>
       <c r="T52" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="53">
@@ -12776,7 +12776,7 @@
         <v>4.101</v>
       </c>
       <c r="T53" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="54">
@@ -12823,7 +12823,7 @@
         <v>11.099</v>
       </c>
       <c r="T54" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="55">
@@ -12879,7 +12879,7 @@
         <v>8.986</v>
       </c>
       <c r="T55" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="56">
@@ -12926,7 +12926,7 @@
         <v>7.214</v>
       </c>
       <c r="T56" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="57">
@@ -12973,7 +12973,7 @@
         <v>3.098</v>
       </c>
       <c r="T57" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="58">
@@ -13029,7 +13029,7 @@
         <v>9.666</v>
       </c>
       <c r="T58" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="59">
@@ -13085,7 +13085,7 @@
         <v>3.457</v>
       </c>
       <c r="T59" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="60">
@@ -13135,7 +13135,7 @@
         <v>1.1</v>
       </c>
       <c r="T60" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="61">
@@ -13191,7 +13191,7 @@
         <v>4.359</v>
       </c>
       <c r="T61" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="62">
@@ -13241,7 +13241,7 @@
         <v>2.044</v>
       </c>
       <c r="T62" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="63">
@@ -13288,7 +13288,7 @@
         <v>1.957</v>
       </c>
       <c r="T63" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="64">
@@ -13338,7 +13338,7 @@
         <v>4.942</v>
       </c>
       <c r="T64" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="65">
@@ -13385,7 +13385,7 @@
         <v>7.482</v>
       </c>
       <c r="T65" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="66">
@@ -13441,7 +13441,7 @@
         <v>4.644</v>
       </c>
       <c r="T66" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="67">
@@ -13497,7 +13497,7 @@
         <v>5.225</v>
       </c>
       <c r="T67" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="68">
@@ -13553,7 +13553,7 @@
         <v>3.028</v>
       </c>
       <c r="T68" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="69">
@@ -13615,7 +13615,7 @@
         <v>3.759</v>
       </c>
       <c r="T69" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="70">
@@ -13662,7 +13662,7 @@
         <v>3.988</v>
       </c>
       <c r="T70" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="71">
@@ -13718,7 +13718,7 @@
         <v>4.7</v>
       </c>
       <c r="T71" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="72">
@@ -13765,7 +13765,7 @@
         <v>3.709</v>
       </c>
       <c r="T72" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="73">
@@ -13827,7 +13827,7 @@
         <v>2056.881</v>
       </c>
       <c r="T73" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="74">
@@ -13883,7 +13883,7 @@
         <v>7.232</v>
       </c>
       <c r="T74" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="75">
@@ -13933,7 +13933,7 @@
         <v>0.232</v>
       </c>
       <c r="T75" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="76">
@@ -13983,7 +13983,7 @@
         <v>3.988</v>
       </c>
       <c r="T76" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="77">
@@ -14039,7 +14039,7 @@
         <v>175.514</v>
       </c>
       <c r="T77" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="78">
@@ -14089,7 +14089,7 @@
         <v>0.232</v>
       </c>
       <c r="T78" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="79">
@@ -14139,7 +14139,7 @@
         <v>0.238</v>
       </c>
       <c r="T79" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="80">
@@ -14186,7 +14186,7 @@
         <v>22.956</v>
       </c>
       <c r="T80" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="81">
@@ -14236,7 +14236,7 @@
         <v>14.437</v>
       </c>
       <c r="T81" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="82">
@@ -14283,7 +14283,7 @@
         <v>23.583</v>
       </c>
       <c r="T82" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="83">
@@ -14333,7 +14333,7 @@
         <v>14.437</v>
       </c>
       <c r="T83" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="84">
@@ -14389,7 +14389,7 @@
         <v>2.152</v>
       </c>
       <c r="T84" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="85">
@@ -14436,7 +14436,7 @@
         <v>23.583</v>
       </c>
       <c r="T85" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="86">
@@ -14483,7 +14483,7 @@
         <v>0.126</v>
       </c>
       <c r="T86" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="87">
@@ -14530,7 +14530,7 @@
         <v>1.504</v>
       </c>
       <c r="T87" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="88">
@@ -14577,7 +14577,7 @@
         <v>15.823</v>
       </c>
       <c r="T88" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="89">
@@ -14624,7 +14624,7 @@
         <v>1.952</v>
       </c>
       <c r="T89" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="90">
@@ -14671,7 +14671,7 @@
         <v>2.639</v>
       </c>
       <c r="T90" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="91">
@@ -14727,7 +14727,7 @@
         <v>5.701</v>
       </c>
       <c r="T91" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="92">
@@ -14774,7 +14774,7 @@
         <v>4.998</v>
       </c>
       <c r="T92" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="93">
@@ -14821,7 +14821,7 @@
         <v>3.535</v>
       </c>
       <c r="T93" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="94">
@@ -14868,7 +14868,7 @@
         <v>1.618</v>
       </c>
       <c r="T94" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="95">
@@ -14915,7 +14915,7 @@
         <v>3.998</v>
       </c>
       <c r="T95" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="96">
@@ -14962,7 +14962,7 @@
         <v>11.408</v>
       </c>
       <c r="T96" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="97">
@@ -15018,7 +15018,7 @@
         <v>11.895</v>
       </c>
       <c r="T97" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="98">
@@ -15065,7 +15065,7 @@
         <v>2.219</v>
       </c>
       <c r="T98" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="99">
@@ -15112,7 +15112,7 @@
         <v>4.377</v>
       </c>
       <c r="T99" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="100">
@@ -15159,7 +15159,7 @@
         <v>2.278</v>
       </c>
       <c r="T100" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="101">
@@ -15209,7 +15209,7 @@
         <v>1.363</v>
       </c>
       <c r="T101" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="102">
@@ -15256,7 +15256,7 @@
         <v>4.379</v>
       </c>
       <c r="T102" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="103">
@@ -15303,7 +15303,7 @@
         <v>4.377</v>
       </c>
       <c r="T103" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="104">
@@ -15350,7 +15350,7 @@
         <v>5.777</v>
       </c>
       <c r="T104" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="105">
@@ -15400,7 +15400,7 @@
         <v>8.469</v>
       </c>
       <c r="T105" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="106">
@@ -15450,7 +15450,7 @@
         <v>2.711</v>
       </c>
       <c r="T106" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="107">
@@ -15506,7 +15506,7 @@
         <v>4.561</v>
       </c>
       <c r="T107" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="108">
@@ -15556,7 +15556,7 @@
         <v>3.627</v>
       </c>
       <c r="T108" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="109">
@@ -15612,7 +15612,7 @@
         <v>0.802</v>
       </c>
       <c r="T109" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="110">
@@ -15668,7 +15668,7 @@
         <v>6.988</v>
       </c>
       <c r="T110" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="111">
@@ -15724,7 +15724,7 @@
         <v>0.437</v>
       </c>
       <c r="T111" t="str">
-        <v>⚠️ Slightly High</v>
+        <v>✅ Within Allocation</v>
       </c>
     </row>
     <row r="112">
@@ -15786,7 +15786,7 @@
         <v>4.477</v>
       </c>
       <c r="T112" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="113">
@@ -15842,7 +15842,7 @@
         <v>0.146</v>
       </c>
       <c r="T113" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="114">
@@ -15898,7 +15898,7 @@
         <v>1.978</v>
       </c>
       <c r="T114" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="115">
@@ -15954,7 +15954,7 @@
         <v>6.707</v>
       </c>
       <c r="T115" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="116">
@@ -16010,7 +16010,7 @@
         <v>6.707</v>
       </c>
       <c r="T116" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="117">
@@ -16066,7 +16066,7 @@
         <v>6.707</v>
       </c>
       <c r="T117" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="118">
@@ -16122,7 +16122,7 @@
         <v>4.788</v>
       </c>
       <c r="T118" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="119">
@@ -16178,7 +16178,7 @@
         <v>4.788</v>
       </c>
       <c r="T119" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="120">
@@ -16225,7 +16225,7 @@
         <v>69.611</v>
       </c>
       <c r="T120" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="121">
@@ -16272,7 +16272,7 @@
         <v>69.333</v>
       </c>
       <c r="T121" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -16424,7 +16424,7 @@
         <v>0.043</v>
       </c>
       <c r="T2" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="3">
@@ -16480,7 +16480,7 @@
         <v>4.036</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -16536,7 +16536,7 @@
         <v>4.036</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -16598,7 +16598,7 @@
         <v>4.477</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -16741,7 +16741,7 @@
         <v>7.482</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -16892,7 +16892,7 @@
         <v>0.802</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -17058,7 +17058,7 @@
         <v>9.211</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -17105,7 +17105,7 @@
         <v>3.886</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -17161,7 +17161,7 @@
         <v>0.534</v>
       </c>
       <c r="T4" t="str">
-        <v>⚠️ Slightly High</v>
+        <v>⚠️ Slightly Over Budget</v>
       </c>
     </row>
     <row r="5">
@@ -17208,7 +17208,7 @@
         <v>2.618</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -17264,7 +17264,7 @@
         <v>8.373</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -17320,7 +17320,7 @@
         <v>8.307</v>
       </c>
       <c r="T7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="8">
@@ -17376,7 +17376,7 @@
         <v>5.828</v>
       </c>
       <c r="T8" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="9">
@@ -17432,7 +17432,7 @@
         <v>10.169</v>
       </c>
       <c r="T9" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="10">
@@ -17488,7 +17488,7 @@
         <v>5.916</v>
       </c>
       <c r="T10" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="11">
@@ -17544,7 +17544,7 @@
         <v>3.367</v>
       </c>
       <c r="T11" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="12">
@@ -17591,7 +17591,7 @@
         <v>2.974</v>
       </c>
       <c r="T12" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="13">
@@ -17647,7 +17647,7 @@
         <v>7.629</v>
       </c>
       <c r="T13" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="14">
@@ -17694,7 +17694,7 @@
         <v>6.453</v>
       </c>
       <c r="T14" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="15">
@@ -17741,7 +17741,7 @@
         <v>4.484</v>
       </c>
       <c r="T15" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="16">
@@ -17788,7 +17788,7 @@
         <v>4.867</v>
       </c>
       <c r="T16" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="17">
@@ -17844,7 +17844,7 @@
         <v>7.884</v>
       </c>
       <c r="T17" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="18">
@@ -17891,7 +17891,7 @@
         <v>4.641</v>
       </c>
       <c r="T18" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="19">
@@ -17947,7 +17947,7 @@
         <v>6.857</v>
       </c>
       <c r="T19" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="20">
@@ -18003,7 +18003,7 @@
         <v>4.101</v>
       </c>
       <c r="T20" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="21">
@@ -18050,7 +18050,7 @@
         <v>11.099</v>
       </c>
       <c r="T21" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="22">
@@ -18106,7 +18106,7 @@
         <v>8.986</v>
       </c>
       <c r="T22" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="23">
@@ -18153,7 +18153,7 @@
         <v>7.214</v>
       </c>
       <c r="T23" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="24">
@@ -18200,7 +18200,7 @@
         <v>1.957</v>
       </c>
       <c r="T24" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="25">
@@ -18250,7 +18250,7 @@
         <v>4.942</v>
       </c>
       <c r="T25" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="26">
@@ -18297,7 +18297,7 @@
         <v>7.482</v>
       </c>
       <c r="T26" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="27">
@@ -18344,7 +18344,7 @@
         <v>3.988</v>
       </c>
       <c r="T27" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="28">
@@ -18400,7 +18400,7 @@
         <v>4.7</v>
       </c>
       <c r="T28" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="29">
@@ -18447,7 +18447,7 @@
         <v>3.709</v>
       </c>
       <c r="T29" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="30">
@@ -18509,7 +18509,7 @@
         <v>2056.881</v>
       </c>
       <c r="T30" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="31">
@@ -18565,7 +18565,7 @@
         <v>7.232</v>
       </c>
       <c r="T31" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="32">
@@ -18615,7 +18615,7 @@
         <v>0.232</v>
       </c>
       <c r="T32" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="33">
@@ -18665,7 +18665,7 @@
         <v>3.988</v>
       </c>
       <c r="T33" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="34">
@@ -18721,7 +18721,7 @@
         <v>175.514</v>
       </c>
       <c r="T34" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="35">
@@ -18771,7 +18771,7 @@
         <v>0.232</v>
       </c>
       <c r="T35" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="36">
@@ -18821,7 +18821,7 @@
         <v>0.238</v>
       </c>
       <c r="T36" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="37">
@@ -18868,7 +18868,7 @@
         <v>22.956</v>
       </c>
       <c r="T37" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="38">
@@ -18918,7 +18918,7 @@
         <v>14.437</v>
       </c>
       <c r="T38" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="39">
@@ -18965,7 +18965,7 @@
         <v>23.583</v>
       </c>
       <c r="T39" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="40">
@@ -19015,7 +19015,7 @@
         <v>14.437</v>
       </c>
       <c r="T40" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="41">
@@ -19071,7 +19071,7 @@
         <v>2.152</v>
       </c>
       <c r="T41" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="42">
@@ -19118,7 +19118,7 @@
         <v>23.583</v>
       </c>
       <c r="T42" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="43">
@@ -19165,7 +19165,7 @@
         <v>0.126</v>
       </c>
       <c r="T43" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="44">
@@ -19212,7 +19212,7 @@
         <v>1.504</v>
       </c>
       <c r="T44" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="45">
@@ -19259,7 +19259,7 @@
         <v>15.823</v>
       </c>
       <c r="T45" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="46">
@@ -19306,7 +19306,7 @@
         <v>1.952</v>
       </c>
       <c r="T46" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="47">
@@ -19353,7 +19353,7 @@
         <v>2.639</v>
       </c>
       <c r="T47" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="48">
@@ -19409,7 +19409,7 @@
         <v>5.701</v>
       </c>
       <c r="T48" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="49">
@@ -19456,7 +19456,7 @@
         <v>4.998</v>
       </c>
       <c r="T49" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="50">
@@ -19503,7 +19503,7 @@
         <v>3.535</v>
       </c>
       <c r="T50" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="51">
@@ -19550,7 +19550,7 @@
         <v>1.618</v>
       </c>
       <c r="T51" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="52">
@@ -19597,7 +19597,7 @@
         <v>3.998</v>
       </c>
       <c r="T52" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="53">
@@ -19644,7 +19644,7 @@
         <v>11.408</v>
       </c>
       <c r="T53" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="54">
@@ -19700,7 +19700,7 @@
         <v>11.895</v>
       </c>
       <c r="T54" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="55">
@@ -19747,7 +19747,7 @@
         <v>2.219</v>
       </c>
       <c r="T55" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="56">
@@ -19794,7 +19794,7 @@
         <v>4.377</v>
       </c>
       <c r="T56" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="57">
@@ -19841,7 +19841,7 @@
         <v>2.278</v>
       </c>
       <c r="T57" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="58">
@@ -19891,7 +19891,7 @@
         <v>1.363</v>
       </c>
       <c r="T58" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="59">
@@ -19938,7 +19938,7 @@
         <v>4.379</v>
       </c>
       <c r="T59" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="60">
@@ -19985,7 +19985,7 @@
         <v>4.377</v>
       </c>
       <c r="T60" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="61">
@@ -20032,7 +20032,7 @@
         <v>5.777</v>
       </c>
       <c r="T61" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="62">
@@ -20082,7 +20082,7 @@
         <v>8.469</v>
       </c>
       <c r="T62" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="63">
@@ -20132,7 +20132,7 @@
         <v>2.711</v>
       </c>
       <c r="T63" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="64">
@@ -20188,7 +20188,7 @@
         <v>4.561</v>
       </c>
       <c r="T64" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="65">
@@ -20238,7 +20238,7 @@
         <v>3.627</v>
       </c>
       <c r="T65" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="66">
@@ -20294,7 +20294,7 @@
         <v>0.802</v>
       </c>
       <c r="T66" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="67">
@@ -20350,7 +20350,7 @@
         <v>6.988</v>
       </c>
       <c r="T67" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="68">
@@ -20406,7 +20406,7 @@
         <v>0.437</v>
       </c>
       <c r="T68" t="str">
-        <v>⚠️ Slightly High</v>
+        <v>✅ Within Allocation</v>
       </c>
     </row>
     <row r="69">
@@ -20468,7 +20468,7 @@
         <v>4.477</v>
       </c>
       <c r="T69" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="70">
@@ -20524,7 +20524,7 @@
         <v>0.146</v>
       </c>
       <c r="T70" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="71">
@@ -20580,7 +20580,7 @@
         <v>1.978</v>
       </c>
       <c r="T71" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="72">
@@ -20636,7 +20636,7 @@
         <v>6.707</v>
       </c>
       <c r="T72" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="73">
@@ -20692,7 +20692,7 @@
         <v>6.707</v>
       </c>
       <c r="T73" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="74">
@@ -20748,7 +20748,7 @@
         <v>6.707</v>
       </c>
       <c r="T74" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="75">
@@ -20804,7 +20804,7 @@
         <v>4.788</v>
       </c>
       <c r="T75" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="76">
@@ -20860,7 +20860,7 @@
         <v>4.788</v>
       </c>
       <c r="T76" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="77">
@@ -20907,7 +20907,7 @@
         <v>69.611</v>
       </c>
       <c r="T77" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="78">
@@ -20954,7 +20954,7 @@
         <v>69.333</v>
       </c>
       <c r="T78" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -21100,7 +21100,7 @@
         <v>0.058</v>
       </c>
       <c r="T2" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="3">
@@ -21150,7 +21150,7 @@
         <v>4.195</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -21197,7 +21197,7 @@
         <v>6.952</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -21244,7 +21244,7 @@
         <v>3.381</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -21291,7 +21291,7 @@
         <v>3.547</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -21338,7 +21338,7 @@
         <v>3.006</v>
       </c>
       <c r="T7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="8">
@@ -21385,7 +21385,7 @@
         <v>2.335</v>
       </c>
       <c r="T8" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="9">
@@ -21435,7 +21435,7 @@
         <v>0.659</v>
       </c>
       <c r="T9" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="10">
@@ -21485,7 +21485,7 @@
         <v>2.609</v>
       </c>
       <c r="T10" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="11">
@@ -21541,7 +21541,7 @@
         <v>3.142</v>
       </c>
       <c r="T11" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="12">
@@ -21597,7 +21597,7 @@
         <v>6.623</v>
       </c>
       <c r="T12" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="13">
@@ -21644,7 +21644,7 @@
         <v>3.381</v>
       </c>
       <c r="T13" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="14">
@@ -21691,7 +21691,7 @@
         <v>5.231</v>
       </c>
       <c r="T14" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="15">
@@ -21747,7 +21747,7 @@
         <v>1.977</v>
       </c>
       <c r="T15" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="16">
@@ -21803,7 +21803,7 @@
         <v>1.748</v>
       </c>
       <c r="T16" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="17">
@@ -21859,7 +21859,7 @@
         <v>4.317</v>
       </c>
       <c r="T17" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="18">
@@ -21909,7 +21909,7 @@
         <v>2.512</v>
       </c>
       <c r="T18" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="19">
@@ -21959,7 +21959,7 @@
         <v>2.609</v>
       </c>
       <c r="T19" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="20">
@@ -22006,7 +22006,7 @@
         <v>5.436</v>
       </c>
       <c r="T20" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="21">
@@ -22053,7 +22053,7 @@
         <v>3.129</v>
       </c>
       <c r="T21" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="22">
@@ -22109,7 +22109,7 @@
         <v>0.094</v>
       </c>
       <c r="T22" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="23">
@@ -22156,7 +22156,7 @@
         <v>3.098</v>
       </c>
       <c r="T23" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="24">
@@ -22212,7 +22212,7 @@
         <v>9.666</v>
       </c>
       <c r="T24" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="25">
@@ -22268,7 +22268,7 @@
         <v>3.457</v>
       </c>
       <c r="T25" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="26">
@@ -22318,7 +22318,7 @@
         <v>1.1</v>
       </c>
       <c r="T26" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="27">
@@ -22374,7 +22374,7 @@
         <v>4.359</v>
       </c>
       <c r="T27" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="28">
@@ -22424,7 +22424,7 @@
         <v>2.044</v>
       </c>
       <c r="T28" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="29">
@@ -22480,7 +22480,7 @@
         <v>4.644</v>
       </c>
       <c r="T29" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="30">
@@ -22536,7 +22536,7 @@
         <v>5.225</v>
       </c>
       <c r="T30" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="31">
@@ -22592,7 +22592,7 @@
         <v>3.028</v>
       </c>
       <c r="T31" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="32">
@@ -22654,7 +22654,7 @@
         <v>3.759</v>
       </c>
       <c r="T32" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -22797,7 +22797,7 @@
         <v>4.879</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -22853,7 +22853,7 @@
         <v>0.043</v>
       </c>
       <c r="T3" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="4">
@@ -22900,7 +22900,7 @@
         <v>5.6</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -22947,7 +22947,7 @@
         <v>2.881</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="6">
@@ -23003,7 +23003,7 @@
         <v>1.165</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="7">
@@ -23053,7 +23053,7 @@
         <v>6.14</v>
       </c>
       <c r="T7" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="8">
@@ -23109,7 +23109,7 @@
         <v>4.036</v>
       </c>
       <c r="T8" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="9">
@@ -23165,7 +23165,7 @@
         <v>4.49</v>
       </c>
       <c r="T9" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="10">
@@ -23221,7 +23221,7 @@
         <v>2.681</v>
       </c>
       <c r="T10" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="11">
@@ -23277,7 +23277,7 @@
         <v>4.036</v>
       </c>
       <c r="T11" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="12">
@@ -23333,7 +23333,7 @@
         <v>4.129</v>
       </c>
       <c r="T12" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="13">
@@ -23389,7 +23389,7 @@
         <v>6.735</v>
       </c>
       <c r="T13" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -23541,7 +23541,7 @@
         <v>0.534</v>
       </c>
       <c r="T2" t="str">
-        <v>⚠️ Slightly High</v>
+        <v>⚠️ Slightly Over Budget</v>
       </c>
     </row>
     <row r="3">
@@ -23591,7 +23591,7 @@
         <v>0.232</v>
       </c>
       <c r="T3" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="4">
@@ -23641,7 +23641,7 @@
         <v>0.232</v>
       </c>
       <c r="T4" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="5">
@@ -23691,7 +23691,7 @@
         <v>0.238</v>
       </c>
       <c r="T5" t="str">
-        <v>✅ Excellent</v>
+        <v>🏆 Below Budget — Best</v>
       </c>
     </row>
     <row r="6">
@@ -23738,7 +23738,7 @@
         <v>4.379</v>
       </c>
       <c r="T6" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>
@@ -23884,7 +23884,7 @@
         <v>2.609</v>
       </c>
       <c r="T2" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="3">
@@ -23934,7 +23934,7 @@
         <v>2.609</v>
       </c>
       <c r="T3" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="4">
@@ -23990,7 +23990,7 @@
         <v>3.367</v>
       </c>
       <c r="T4" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
     <row r="5">
@@ -24046,7 +24046,7 @@
         <v>4.101</v>
       </c>
       <c r="T5" t="str">
-        <v>🔴 Above Normal</v>
+        <v>🔴 Over Budget — Investigate</v>
       </c>
     </row>
   </sheetData>

</xml_diff>